<commit_message>
Day 3 and Day 4
</commit_message>
<xml_diff>
--- a/Day1/ml_30_day_progress_tracker.xlsx
+++ b/Day1/ml_30_day_progress_tracker.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ketan\Desktop\ML MODELS\Day1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4B235A-B810-4FEC-9622-AA55548D9322}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13FC376-D283-4E61-9197-0A372DC5B1EC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -370,6 +370,9 @@
                 <c:ptCount val="30"/>
                 <c:pt idx="0">
                   <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2</c:v>
                 </c:pt>
                 <c:pt idx="14">
                   <c:v>0</c:v>
@@ -804,7 +807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H31"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="59.28515625" customWidth="1"/>
@@ -862,7 +865,13 @@
         <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
+        <v>38</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>